<commit_message>
docs(qa): actualizar plantilla de seguimiento de pruebas con cuadros simetricos y filas uniformes
</commit_message>
<xml_diff>
--- a/docs/entregables/Plantilla_Seguimiento_Ejecucion_Pruebas.xlsx
+++ b/docs/entregables/Plantilla_Seguimiento_Ejecucion_Pruebas.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,7 +63,19 @@
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="7">
@@ -99,8 +111,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -179,8 +191,36 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -548,10 +588,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col hidden="1" width="42" customWidth="1" min="3" max="3"/>
     <col hidden="1" width="12" customWidth="1" min="4" max="4"/>
     <col hidden="1" width="25" customWidth="1" min="5" max="5"/>
@@ -561,9 +601,9 @@
     <col hidden="1" width="30" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="25" customWidth="1" min="10" max="10"/>
     <col hidden="1" width="15" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
     <col hidden="1" width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -581,25 +621,28 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Ciclo de Pruebas: Seguimiento de Ejecución — Aceptación</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="B3" s="13" t="n"/>
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>Información para el Seguimiento</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="M3" s="13" t="n"/>
+      <c r="N3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Caso de Prueba</t>
         </is>
@@ -649,17 +692,17 @@
           <t>Dependencias con otros casos de Prueba</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="14" t="inlineStr">
         <is>
           <t>Resultado Obtenido</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="14" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>Última Fecha de Estado</t>
         </is>
@@ -670,13 +713,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>TC-01</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>TC_01_Autenticacion_LoginAsync_AdministradorAutorizado</t>
         </is>
@@ -726,17 +769,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M5" s="12" t="inlineStr">
+      <c r="M5" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -747,13 +790,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>TC-02</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>TC_02_ConsultaReservas_ObtenerPorDiaAsync_FechaEspecifica</t>
         </is>
@@ -803,17 +846,17 @@
           <t>TC-01</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M6" s="12" t="inlineStr">
+      <c r="M6" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
+      <c r="N6" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -824,13 +867,13 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>TC-03</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>TC_03_CreacionYPersistenciaReserva_ReservarAsync</t>
         </is>
@@ -880,17 +923,17 @@
           <t>TC-01</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L7" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M7" s="12" t="inlineStr">
+      <c r="M7" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -901,13 +944,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>TC_04_ReporteRangoFechas_InclusionesYExclusiones</t>
         </is>
@@ -957,17 +1000,17 @@
           <t>TC-01</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="L8" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M8" s="12" t="inlineStr">
+      <c r="M8" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N8" s="11" t="inlineStr">
+      <c r="N8" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -978,13 +1021,13 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>TC-05</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>TC_05_ValidarAnticolision_DisponibilidadService_Y_ReservaService</t>
         </is>
@@ -1034,17 +1077,17 @@
           <t>TC-03</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M9" s="12" t="inlineStr">
+      <c r="M9" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1055,13 +1098,13 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>TC-06</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>TC_06_ValidarCalculoDinamicoTarifaTemporadaAlta_3Noches_X_120</t>
         </is>
@@ -1111,17 +1154,17 @@
           <t>TC-03</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="L10" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M10" s="12" t="inlineStr">
+      <c r="M10" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N10" s="11" t="inlineStr">
+      <c r="N10" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1132,13 +1175,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>TC-07</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>TC_07_ValidarPasswordAsync_VerificacionHashSHA256</t>
         </is>
@@ -1188,17 +1231,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L11" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M11" s="12" t="inlineStr">
+      <c r="M11" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
+      <c r="N11" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1209,13 +1252,13 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TC-08</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>TC_08_RestriccionAccesoAdministrativo_UsuarioSinPermisos</t>
         </is>
@@ -1265,17 +1308,17 @@
           <t>TC-01</t>
         </is>
       </c>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="L12" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M12" s="12" t="inlineStr">
+      <c r="M12" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N12" s="11" t="inlineStr">
+      <c r="N12" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1289,9 +1332,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="L3:O3"/>
     <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1304,10 +1347,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col hidden="1" width="42" customWidth="1" min="3" max="3"/>
     <col hidden="1" width="12" customWidth="1" min="4" max="4"/>
     <col hidden="1" width="25" customWidth="1" min="5" max="5"/>
@@ -1317,9 +1360,9 @@
     <col hidden="1" width="30" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="25" customWidth="1" min="10" max="10"/>
     <col hidden="1" width="15" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
     <col hidden="1" width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -1337,25 +1380,28 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Ciclo de Pruebas: Seguimiento de Ejecución — API</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="B3" s="13" t="n"/>
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>Información para el Seguimiento</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="M3" s="13" t="n"/>
+      <c r="N3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Caso de Prueba</t>
         </is>
@@ -1405,17 +1451,17 @@
           <t>Dependencias con otros casos de Prueba</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="14" t="inlineStr">
         <is>
           <t>Resultado Obtenido</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="14" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>Última Fecha de Estado</t>
         </is>
@@ -1426,13 +1472,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>API-01</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>PostReserva_ConAmbasFechasEnElPasado_Retorna400BadRequest</t>
         </is>
@@ -1482,17 +1528,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M5" s="12" t="inlineStr">
+      <c r="M5" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1503,13 +1549,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>API-02</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>PostReserva_ConFechaEntradaEnElPasado_Retorna400BadRequest</t>
         </is>
@@ -1559,17 +1605,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M6" s="12" t="inlineStr">
+      <c r="M6" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
+      <c r="N6" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1580,13 +1626,13 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>API-03</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>PostReserva_ConFechaEntradaIgualASalida_Retorna400BadRequest</t>
         </is>
@@ -1636,17 +1682,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L7" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M7" s="12" t="inlineStr">
+      <c r="M7" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1657,13 +1703,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>API-04</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>PostReserva_ConFechaEntradaMayorQueSalida_Retorna400BadRequest</t>
         </is>
@@ -1713,17 +1759,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="L8" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M8" s="12" t="inlineStr">
+      <c r="M8" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N8" s="11" t="inlineStr">
+      <c r="N8" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1734,13 +1780,13 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>API-05</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>PostReserva_ConFechasValidas_Retorna200OkYPersisteReserva</t>
         </is>
@@ -1790,17 +1836,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M9" s="12" t="inlineStr">
+      <c r="M9" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1811,13 +1857,13 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>API-06</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>GetDisponibilidad_EnRangoConReservaActiva_ExcluyeHabitacionOcupada</t>
         </is>
@@ -1867,17 +1913,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="L10" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M10" s="12" t="inlineStr">
+      <c r="M10" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N10" s="11" t="inlineStr">
+      <c r="N10" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1888,13 +1934,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>API-07</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>GetDisponibilidad_EnRangoSinConflicto_Retorna200OkYHabitacionDisponible</t>
         </is>
@@ -1944,17 +1990,17 @@
           <t>API-06</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L11" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M11" s="12" t="inlineStr">
+      <c r="M11" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
+      <c r="N11" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -1965,13 +2011,13 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>API-08</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>GetDisponibilidad_HabitacionInactiva_NoSeIncluyeEnDisponibles</t>
         </is>
@@ -2021,17 +2067,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="L12" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M12" s="12" t="inlineStr">
+      <c r="M12" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N12" s="11" t="inlineStr">
+      <c r="N12" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2042,13 +2088,13 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>API-09</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>GetDetalles_ConIdExistente_Retorna200OkYReservaCorrespondiente</t>
         </is>
@@ -2098,17 +2144,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L13" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M13" s="12" t="inlineStr">
+      <c r="M13" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
+      <c r="N13" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2119,13 +2165,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>API-10</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>GetDetalles_ConIdInexistente_Retorna404NotFound</t>
         </is>
@@ -2175,17 +2221,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="L14" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M14" s="12" t="inlineStr">
+      <c r="M14" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N14" s="11" t="inlineStr">
+      <c r="N14" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2196,13 +2242,13 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>API-11</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>GetObtenerPorDia_ConFechaConReservas_Retorna200OkYListaReservas</t>
         </is>
@@ -2252,17 +2298,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L15" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="M15" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="N15" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2273,13 +2319,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>API-12</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>GetObtenerPorDia_ConFechaSinReservas_Retorna200OkYListaVacia</t>
         </is>
@@ -2329,17 +2375,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L16" s="10" t="inlineStr">
+      <c r="L16" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M16" s="12" t="inlineStr">
+      <c r="M16" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N16" s="11" t="inlineStr">
+      <c r="N16" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2350,13 +2396,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>API-13</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>PostCancelarReserva_ActualizaEstadoEnBaseDeDatosInMemory</t>
         </is>
@@ -2406,17 +2452,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L17" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M17" s="12" t="inlineStr">
+      <c r="M17" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N17" s="7" t="inlineStr">
+      <c r="N17" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2427,13 +2473,13 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>API-14</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>PostCancelarReserva_ConIdInexistente_Retorna404NotFound</t>
         </is>
@@ -2483,17 +2529,17 @@
           <t>API-13</t>
         </is>
       </c>
-      <c r="L18" s="10" t="inlineStr">
+      <c r="L18" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M18" s="12" t="inlineStr">
+      <c r="M18" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N18" s="11" t="inlineStr">
+      <c r="N18" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2504,13 +2550,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>API-15</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>PostCrearReserva_EnMismasFechasQueReservaActiva_RechazaPorColision</t>
         </is>
@@ -2560,17 +2606,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L19" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M19" s="12" t="inlineStr">
+      <c r="M19" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
+      <c r="N19" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2581,13 +2627,13 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>API-16</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>PostCrearReserva_PersisteEntidadEnBaseDeDatosInMemory</t>
         </is>
@@ -2637,17 +2683,17 @@
           <t>API-13</t>
         </is>
       </c>
-      <c r="L20" s="10" t="inlineStr">
+      <c r="L20" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M20" s="12" t="inlineStr">
+      <c r="M20" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N20" s="11" t="inlineStr">
+      <c r="N20" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2661,9 +2707,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="L3:O3"/>
     <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2676,10 +2722,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col hidden="1" width="42" customWidth="1" min="3" max="3"/>
     <col hidden="1" width="12" customWidth="1" min="4" max="4"/>
     <col hidden="1" width="25" customWidth="1" min="5" max="5"/>
@@ -2689,9 +2735,9 @@
     <col hidden="1" width="30" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="25" customWidth="1" min="10" max="10"/>
     <col hidden="1" width="15" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
     <col hidden="1" width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -2709,25 +2755,28 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Ciclo de Pruebas: Seguimiento de Ejecución — Unitarias</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="B3" s="13" t="n"/>
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>Información para el Seguimiento</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="M3" s="13" t="n"/>
+      <c r="N3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Caso de Prueba</t>
         </is>
@@ -2777,17 +2826,17 @@
           <t>Dependencias con otros casos de Prueba</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="14" t="inlineStr">
         <is>
           <t>Resultado Obtenido</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="14" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="14" t="inlineStr">
         <is>
           <t>Última Fecha de Estado</t>
         </is>
@@ -2798,13 +2847,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>UT-01</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>FechasValidas_EntradaEnElPasado_RetornaFalse</t>
         </is>
@@ -2854,17 +2903,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M5" s="12" t="inlineStr">
+      <c r="M5" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N5" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2875,13 +2924,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>UT-02</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>FechasValidas_EntradaFuturaYMenorQueSalida_RetornaTrue</t>
         </is>
@@ -2931,17 +2980,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M6" s="12" t="inlineStr">
+      <c r="M6" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
+      <c r="N6" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -2952,13 +3001,13 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>UT-03</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>FechasValidas_EntradaHoyYSalidaManana_RetornaTrue</t>
         </is>
@@ -3008,17 +3057,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L7" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M7" s="12" t="inlineStr">
+      <c r="M7" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3029,13 +3078,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>UT-04</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>FechasValidas_EntradaIgualASalida_RetornaFalse</t>
         </is>
@@ -3085,17 +3134,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="L8" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M8" s="12" t="inlineStr">
+      <c r="M8" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N8" s="11" t="inlineStr">
+      <c r="N8" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3106,13 +3155,13 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>UT-05</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>FechasValidas_EntradaMayorQueSalida_RetornaFalse</t>
         </is>
@@ -3162,17 +3211,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M9" s="12" t="inlineStr">
+      <c r="M9" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N9" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3183,13 +3232,13 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>UT-06</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>FechasValidas_EntradaYSalidaEnElPasado_RetornaFalse</t>
         </is>
@@ -3239,17 +3288,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="L10" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M10" s="12" t="inlineStr">
+      <c r="M10" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N10" s="11" t="inlineStr">
+      <c r="N10" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3260,13 +3309,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>UT-07</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>ObtenerDisponiblesAsync_ConReservaActivaEnConflicto_ExcluyeHabitacionOcupada</t>
         </is>
@@ -3316,17 +3365,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L11" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M11" s="12" t="inlineStr">
+      <c r="M11" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N11" s="7" t="inlineStr">
+      <c r="N11" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3337,13 +3386,13 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>UT-08</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>ObtenerDisponiblesAsync_ConReservaCanceladaEnMismoRango_NoExcluyeHabitacion</t>
         </is>
@@ -3393,17 +3442,17 @@
           <t>UT-07</t>
         </is>
       </c>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="L12" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M12" s="12" t="inlineStr">
+      <c r="M12" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N12" s="11" t="inlineStr">
+      <c r="N12" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3414,13 +3463,13 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>UT-09</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>ObtenerDisponiblesAsync_HabitacionInactiva_NoSeIncluyeEnDisponibles</t>
         </is>
@@ -3470,17 +3519,17 @@
           <t>UT-07</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L13" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M13" s="12" t="inlineStr">
+      <c r="M13" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
+      <c r="N13" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3491,13 +3540,13 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>UT-10</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>ObtenerDisponiblesAsync_ReservaFinalizaElMismoDiaDeEntrada_HabitacionDisponible</t>
         </is>
@@ -3547,17 +3596,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="L14" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M14" s="12" t="inlineStr">
+      <c r="M14" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N14" s="11" t="inlineStr">
+      <c r="N14" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3568,13 +3617,13 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>UT-11</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>ObtenerDisponiblesAsync_ReservaIniciaElMismoDiaDeSalida_HabitacionDisponible</t>
         </is>
@@ -3624,17 +3673,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L15" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="M15" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N15" s="7" t="inlineStr">
+      <c r="N15" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3645,13 +3694,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>UT-12</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>ObtenerDisponiblesAsync_SinReservas_RetornaTodasLasHabitacionesActivas</t>
         </is>
@@ -3701,17 +3750,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L16" s="10" t="inlineStr">
+      <c r="L16" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M16" s="12" t="inlineStr">
+      <c r="M16" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N16" s="11" t="inlineStr">
+      <c r="N16" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3722,13 +3771,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>UT-13</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Actualizar_EstadoModificado_Exitoso</t>
         </is>
@@ -3778,17 +3827,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L17" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M17" s="12" t="inlineStr">
+      <c r="M17" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N17" s="7" t="inlineStr">
+      <c r="N17" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3799,13 +3848,13 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>UT-14</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Disponibilidad_ConConflicto_RetornaFalse</t>
         </is>
@@ -3855,17 +3904,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L18" s="10" t="inlineStr">
+      <c r="L18" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M18" s="12" t="inlineStr">
+      <c r="M18" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N18" s="11" t="inlineStr">
+      <c r="N18" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3876,13 +3925,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>UT-15</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Disponibilidad_SinConflicto_RetornaTrue</t>
         </is>
@@ -3932,17 +3981,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L19" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M19" s="12" t="inlineStr">
+      <c r="M19" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N19" s="7" t="inlineStr">
+      <c r="N19" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -3953,13 +4002,13 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>UT-16</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>Eliminar_PorId_Exitoso</t>
         </is>
@@ -4009,17 +4058,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L20" s="10" t="inlineStr">
+      <c r="L20" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M20" s="12" t="inlineStr">
+      <c r="M20" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N20" s="11" t="inlineStr">
+      <c r="N20" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -4030,13 +4079,13 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>UT-17</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>ObtenerPorDia_FechaValida_RetornaReservas</t>
         </is>
@@ -4086,17 +4135,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L21" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M21" s="12" t="inlineStr">
+      <c r="M21" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
+      <c r="N21" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -4107,13 +4156,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>UT-18</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>ObtenerPorId_IdExistente_RetornaReserva</t>
         </is>
@@ -4163,17 +4212,17 @@
           <t>UT-17</t>
         </is>
       </c>
-      <c r="L22" s="10" t="inlineStr">
+      <c r="L22" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M22" s="12" t="inlineStr">
+      <c r="M22" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N22" s="11" t="inlineStr">
+      <c r="N22" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -4184,13 +4233,13 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>UT-19</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>ObtenerPorId_IdInexistente_RetornaNull</t>
         </is>
@@ -4240,17 +4289,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr">
+      <c r="L23" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M23" s="12" t="inlineStr">
+      <c r="M23" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
+      <c r="N23" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -4261,13 +4310,13 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>UT-20</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>ObtenerTodas_ListaCompleta_RetornaReservas</t>
         </is>
@@ -4317,17 +4366,17 @@
           <t>UT-17</t>
         </is>
       </c>
-      <c r="L24" s="10" t="inlineStr">
+      <c r="L24" s="22" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M24" s="12" t="inlineStr">
+      <c r="M24" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N24" s="11" t="inlineStr">
+      <c r="N24" s="22" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -4338,13 +4387,13 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>UT-21</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>Reservar_DatosValidos_CreaReserva</t>
         </is>
@@ -4394,17 +4443,17 @@
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="L25" s="6" t="inlineStr">
+      <c r="L25" s="18" t="inlineStr">
         <is>
           <t>Aserciones superadas</t>
         </is>
       </c>
-      <c r="M25" s="12" t="inlineStr">
+      <c r="M25" s="19" t="inlineStr">
         <is>
           <t>Exitoso</t>
         </is>
       </c>
-      <c r="N25" s="7" t="inlineStr">
+      <c r="N25" s="18" t="inlineStr">
         <is>
           <t>28/10/2026</t>
         </is>
@@ -4418,9 +4467,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="L3:O3"/>
     <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>